<commit_message>
test(overlap_reviewer): sparse injects — 3 leaks, 1 nonsense, 3 wrong matches
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/overlap_reviewer/testdata/test.1175.injected.xlsx
+++ b/overlap_reviewer/testdata/test.1175.injected.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ich hab dich nie gezwungen, ihn zu verlassen.</t>
+          <t>hast – Ich hab dich nie gezwungen, ihn zu verlassen.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Wo ist Ed?</t>
+          <t>Wo ist das Sofa?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -856,22 +856,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>STEDE</t>
+          <t>BLACKBEARD</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ed!</t>
+          <t>Stede!</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>00:01:15:16</t>
+          <t>00:01:08:11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>00:01:16:00</t>
+          <t>00:01:11:17</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Er hat mich angefurzt.</t>
+          <t>Mann! Er hat mich angefurzt.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1696,22 +1696,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ROACH</t>
+          <t>BLACK PETE</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Halt die Klappe!</t>
+          <t>Halt's Maul! Es reicht!</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00:02:25:07</t>
+          <t>00:02:26:19</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>00:02:26:15</t>
+          <t>00:02:28:03</t>
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
@@ -2620,27 +2620,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Das ist der Schwede.</t>
+          <t>du? Das ist der Schwede.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>OLUWANDE</t>
+          <t>SCHWEDE</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Das ist der Schwede.</t>
+          <t>Ich bin der Schwede.</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>00:03:25:11</t>
+          <t>00:03:26:03</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>00:03:26:02</t>
+          <t>00:03:26:22</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>

</xml_diff>

<commit_message>
test(overlap_reviewer): mark injects red + INJECTED-ERROR; keep only Du unglaubliche
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/overlap_reviewer/testdata/test.1175.injected.xlsx
+++ b/overlap_reviewer/testdata/test.1175.injected.xlsx
@@ -26,12 +26,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCCC"/>
+        <bgColor rgb="00FFCCCC"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +464,11 @@
           <t>NOT_MATCHED</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>INJECTED-ERROR</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -494,7 +506,6 @@
           <t>00:00:28:06</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -532,7 +543,6 @@
           <t>00:00:30:02</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -570,7 +580,6 @@
           <t>00:00:31:19</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -608,45 +617,49 @@
           <t>00:00:35:12</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>00:00:40:16</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>00:00:42:10</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>hast – Ich hab dich nie gezwungen, ihn zu verlassen.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>IZZY</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Ich hab dich nie gezwungen, ihn zu verlassen. .. Das hast du von allein getan.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>00:00:40:16</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>00:00:42:10</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>TEXT_LEAK: Wort „hast“ vom vorherigen STEDE-Segment klebt am IZZY-Satz (mit anderem Satzzeichen „–“).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -684,7 +697,6 @@
           <t>00:00:44:14</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -722,83 +734,92 @@
           <t>00:00:55:17</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>00:00:56:08</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>00:00:57:01</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Wo ist das Sofa?</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>STEDE</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Wo ist er? .. Wo ist Ed?</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>00:00:56:08</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>00:00:57:04</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>NONSENSE: Sehr nahe am vorherigen Segment „Wo ist er?“ — „Wo ist das Sofa?“ ergibt im Kontext (Suche nach Ed) keinen Sinn.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>00:01:01:06</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>00:01:06:09</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Du unglaubliche Muschi.</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Du unglaubliche.</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>IZZY</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Du unglaublicher . Kackvogel.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>00:01:01:06</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>00:01:06:12</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>ASR/SPLIT: Nur „Du unglaubliche.“ belassen — „Muschi“ entfernt (kein doppelter Anfang „Du unglaubliche … Muschi“). Match bleibt Kackvogel-Zeile.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -836,45 +857,49 @@
           <t>00:01:11:17</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>00:01:15:17</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>00:01:16:00</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Ed!</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>BLACKBEARD</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Stede!</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>00:01:08:11</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>00:01:11:17</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr"/>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>SPEAKER_WRONG: Dialog „Ed!“ behält, aber MATCHED-TEXT/SOURCE/REF fälschlich von vorherigem BLACKBEARD-„Stede!“-Segment übernommen.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -912,7 +937,6 @@
           <t>00:01:18:18</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -950,7 +974,6 @@
           <t>00:01:21:07</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -988,7 +1011,6 @@
           <t>00:01:29:09</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1026,7 +1048,6 @@
           <t>00:01:36:24</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1106,7 +1127,6 @@
           <t>00:01:53:04</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1144,7 +1164,6 @@
           <t>00:01:55:10</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1182,7 +1201,6 @@
           <t>00:01:59:10</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1220,7 +1238,6 @@
           <t>00:02:01:21</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1258,7 +1275,6 @@
           <t>00:02:03:17</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1296,7 +1312,6 @@
           <t>00:02:08:15</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1334,7 +1349,6 @@
           <t>00:02:09:11</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1372,7 +1386,6 @@
           <t>00:02:10:08</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1410,7 +1423,6 @@
           <t>00:02:11:18</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1448,7 +1460,6 @@
           <t>00:02:13:10</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1486,7 +1497,6 @@
           <t>00:02:14:06</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1524,7 +1534,6 @@
           <t>00:02:15:09</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1562,7 +1571,6 @@
           <t>00:02:20:04</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1600,7 +1608,6 @@
           <t>00:02:21:13</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1638,83 +1645,92 @@
           <t>00:02:23:23</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>00:02:24:03</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="1" t="inlineStr">
         <is>
           <t>00:02:25:03</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>Mann! Er hat mich angefurzt.</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>STEDE</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Er hat mich angefurzt.</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>00:02:24:02</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="1" t="inlineStr">
         <is>
           <t>00:02:25:05</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" s="1" t="inlineStr"/>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>TEXT_LEAK: Wort „Mann“ vom vorherigen BUTTONS-Segment klebt am STEDE-Satz (Satzzeichen „!“ statt „?“).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>00:02:25:07</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
         <is>
           <t>00:02:26:11</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>Halt die Klappe!</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>BLACK PETE</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Halt's Maul! Es reicht!</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>00:02:26:19</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="1" t="inlineStr">
         <is>
           <t>00:02:28:03</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" s="1" t="inlineStr"/>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>SPEAKER_WRONG: Dialog „Halt die Klappe!“ (war ROACH), aber MATCHED-TEXT/SOURCE/REF fälschlich vom nächsten BLACK-PETE-Segment übernommen.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1752,7 +1768,6 @@
           <t>00:02:28:03</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1832,7 +1847,6 @@
           <t>00:02:30:17</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1870,7 +1884,6 @@
           <t>00:02:35:01</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1950,7 +1963,6 @@
           <t>00:02:39:08</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1988,7 +2000,6 @@
           <t>00:02:40:23</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2111,7 +2122,6 @@
           <t>00:02:46:11</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2149,7 +2159,6 @@
           <t>00:02:48:19</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2187,7 +2196,6 @@
           <t>00:02:53:23</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2225,7 +2233,6 @@
           <t>00:02:55:12</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2263,7 +2270,6 @@
           <t>00:03:02:14</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2301,7 +2307,6 @@
           <t>00:03:06:09</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2339,7 +2344,6 @@
           <t>00:03:13:06</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2377,7 +2381,6 @@
           <t>00:03:14:16</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2415,7 +2418,6 @@
           <t>00:03:17:03</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2453,7 +2455,6 @@
           <t>00:03:18:17</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2491,7 +2492,6 @@
           <t>00:03:20:17</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2529,7 +2529,6 @@
           <t>00:03:22:14</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2567,7 +2566,6 @@
           <t>00:03:23:17</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2605,45 +2603,49 @@
           <t>00:03:25:10</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="1" t="inlineStr">
         <is>
           <t>00:03:25:11</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="1" t="inlineStr">
         <is>
           <t>00:03:26:02</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="1" t="inlineStr">
         <is>
           <t>du? Das ist der Schwede.</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="1" t="inlineStr">
         <is>
           <t>SCHWEDE</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="1" t="inlineStr">
         <is>
           <t>Ich bin der Schwede.</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="1" t="inlineStr">
         <is>
           <t>00:03:26:03</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="1" t="inlineStr">
         <is>
           <t>00:03:26:22</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
+      <c r="H58" s="1" t="inlineStr"/>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>TEXT_LEAK: Wort „du“ vom vorherigen STEDE-Segment klebt am OLUWANDE-Satz („?“); zusätzlich SPEAKER_WRONG (siehe Match). SPEAKER_WRONG: MATCHED-TEXT/SOURCE/REF fälschlich vom nächsten SCHWEDE-Segment („Ich bin der Schwede.“) übernommen.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2681,7 +2683,6 @@
           <t>00:03:26:22</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2719,7 +2720,6 @@
           <t>00:03:29:24</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2757,7 +2757,6 @@
           <t>00:03:31:01</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2795,7 +2794,6 @@
           <t>00:03:32:11</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2833,7 +2831,6 @@
           <t>00:03:32:22</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2871,7 +2868,6 @@
           <t>00:03:35:14</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2953,7 +2949,6 @@
           <t>00:03:39:14</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2991,7 +2986,6 @@
           <t>00:03:44:09</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3029,7 +3023,6 @@
           <t>00:03:47:14</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3067,7 +3060,6 @@
           <t>00:03:49:03</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3148,7 +3140,6 @@
           <t>00:03:53:02</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3186,7 +3177,6 @@
           <t>00:03:54:08</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3224,7 +3214,6 @@
           <t>00:03:56:21</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3262,7 +3251,6 @@
           <t>00:03:58:17</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3300,7 +3288,6 @@
           <t>00:03:59:15</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3338,7 +3325,6 @@
           <t>00:04:01:17</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3376,7 +3362,6 @@
           <t>00:04:04:09</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3414,7 +3399,6 @@
           <t>00:04:06:00</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3452,7 +3436,6 @@
           <t>00:04:07:05</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3490,7 +3473,6 @@
           <t>00:04:13:12</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3528,7 +3510,6 @@
           <t>00:04:14:12</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3566,7 +3547,6 @@
           <t>00:04:15:14</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3604,7 +3584,6 @@
           <t>00:04:17:09</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3642,7 +3621,6 @@
           <t>00:04:18:06</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3680,7 +3658,6 @@
           <t>00:04:20:02</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3718,7 +3695,6 @@
           <t>00:04:20:24</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3756,7 +3732,6 @@
           <t>00:04:22:07</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3794,7 +3769,6 @@
           <t>00:04:25:14</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3832,7 +3806,6 @@
           <t>00:04:26:04</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3870,7 +3843,6 @@
           <t>00:04:27:22</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3950,7 +3922,6 @@
           <t>00:04:34:05</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3988,7 +3959,6 @@
           <t>00:04:36:04</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4026,7 +3996,6 @@
           <t>00:04:37:17</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4064,7 +4033,6 @@
           <t>00:04:38:22</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4102,7 +4070,6 @@
           <t>00:04:39:21</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4140,7 +4107,6 @@
           <t>00:04:41:07</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4178,7 +4144,6 @@
           <t>00:04:42:20</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4216,7 +4181,6 @@
           <t>00:04:43:08</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4254,7 +4218,6 @@
           <t>00:04:44:21</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4292,7 +4255,6 @@
           <t>00:04:45:23</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(overlap_reviewer): overlap-chaos block with wrong roles/text + NOT_MATCHED
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/overlap_reviewer/testdata/test.1175.injected.xlsx
+++ b/overlap_reviewer/testdata/test.1175.injected.xlsx
@@ -817,7 +817,7 @@
       <c r="H10" s="1" t="inlineStr"/>
       <c r="I10" s="1" t="inlineStr">
         <is>
-          <t>ASR/SPLIT: Nur „Du unglaubliche.“ belassen — „Muschi“ entfernt (kein doppelter Anfang „Du unglaubliche … Muschi“). Match bleibt Kackvogel-Zeile.</t>
+          <t>ASR/SPLIT: Nur „Du unglaubliche.“ belassen — „Muschi“ entfernt (kein doppelter Anfang). Match bleibt Kackvogel-Zeile.</t>
         </is>
       </c>
     </row>
@@ -1702,186 +1702,193 @@
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>Halt die Klappe!</t>
+          <t>Halt die Klappe Ed oh Ed die Nacht!</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>BLACK PETE</t>
+          <t>STEDE</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>Halt's Maul! Es reicht!</t>
+          <t>Es ist noch da. Es ist 'ne Wand aus Gestank.</t>
         </is>
       </c>
       <c r="F34" s="1" t="inlineStr">
         <is>
-          <t>00:02:26:19</t>
+          <t>00:02:28:10</t>
         </is>
       </c>
       <c r="G34" s="1" t="inlineStr">
         <is>
-          <t>00:02:28:03</t>
+          <t>00:02:29:01</t>
         </is>
       </c>
       <c r="H34" s="1" t="inlineStr"/>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>SPEAKER_WRONG: Dialog „Halt die Klappe!“ (war ROACH), aber MATCHED-TEXT/SOURCE/REF fälschlich vom nächsten BLACK-PETE-Segment übernommen.</t>
+          <t>OVERLAP-CHAOS / SPEAKER_WRONG+TEXT: Dialog mischt ROACH+PETE; fälschlich SOURCE=STEDE und MATCHED-TEXT=Stede-Gestank-Zeile.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="1" t="inlineStr">
         <is>
           <t>00:02:26:20</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
         <is>
           <t>00:02:27:15</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Ach, Schnauze!</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>Schnauze Wand Gestank</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>BUTTONS</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>Kannst du die Schnauze halten, Mann?</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>00:02:22:02</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>00:02:23:23</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr"/>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>OVERLAP-CHAOS / SPEAKER_WRONG+TEXT: „Schnauze Wand Gestank“; fälschlich SOURCE=BUTTONS + Buttons-MATCHED-TEXT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>00:02:28:10</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>00:02:28:24</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>Es ist noch da irgendwie die Klappe</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr"/>
+      <c r="E36" s="1" t="inlineStr"/>
+      <c r="F36" s="1" t="inlineStr"/>
+      <c r="G36" s="1" t="inlineStr"/>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>[Original ohne Transkript-Match] (Script-Zeile #28) Original: 00:02:24:22 – 00:02:28:15 | BUTTONS: Schnauze, Mann! | Platzierung: nicht prüfbar (kein Refine-Zeitcode, Drehbuch-Matcher fehlt oder keine Zeile) || [Original ohne Transkript-Match] (Script-Zeile #29) Original: 00:02:28:10 – 00:02:31:02 | STEDE: Es ist noch da. Es ist 'ne Wand aus Gestank. | Platzierung: nicht prüfbar (kein Refine-Zeitcode, Drehbuch-Matcher fehlt oder keine Zeile)</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>OVERLAP-CHAOS / UNMATCHED: STEDE ohne Match (SOURCE/MATCHED/REF leer); echtes Original in NOT_MATCHED — am Original orientieren/korrigieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>00:02:29:06</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>00:02:30:16</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Es ist eine Wand aus Ed oh Ed Gestöhne</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
         <is>
           <t>BLACK PETE</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Halt's Maul! Es reicht!</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>00:02:26:19</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>00:02:28:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>00:02:28:10</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>00:02:28:24</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Es ist noch da.</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>STEDE</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Es ist noch da. Es ist 'ne Wand aus Gestank.</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>00:02:28:10</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>00:02:29:01</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>[Original ohne Transkript-Match] (Script-Zeile #28) Original: 00:02:24:22 – 00:02:28:15 | BUTTONS: Schnauze, Mann! | Platzierung: nicht prüfbar (kein Refine-Zeitcode, Drehbuch-Matcher fehlt oder keine Zeile)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>00:02:29:06</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>00:02:30:16</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Es ist eine Wand ausgestankt.</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>STEDE</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Es ist noch da. Es ist 'ne Wand aus Gestank.</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>00:02:29:06</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>00:02:30:17</t>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Kann nicht schlimmer sein als Ihr Ed, oh Ed"-Gestöhne die ganze Nacht."</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>00:02:30:19</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>00:02:35:01</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="inlineStr"/>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>OVERLAP-CHAOS / SPEAKER_WRONG+TEXT: Gestank+Pete vermischt; fälschlich SOURCE=BLACK PETE + Pete-MATCHED-TEXT.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="1" t="inlineStr">
         <is>
           <t>00:02:30:19</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="1" t="inlineStr">
         <is>
           <t>00:02:34:13</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Kann nicht schlimmer sein als sein Et-O-Et-Gestöhne die ganze Nacht.</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>BLACK PETE</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Kann nicht schlimmer sein als Ihr Ed, oh Ed"-Gestöhne die ganze Nacht."</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>00:02:30:19</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>00:02:35:01</t>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Kann nicht schlimmer Halt die Klappe die ganze Nacht</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>ROACH</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>Halt die Klappe!</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr">
+        <is>
+          <t>00:02:25:07</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>00:02:26:15</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr"/>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>OVERLAP-CHAOS / SPEAKER_WRONG+TEXT: PETE-Satz mit ROACH-Leak; fälschlich SOURCE=ROACH + MATCHED-TEXT „Halt die Klappe!“.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: append Korean/exotic name ASR errors with matching original cues
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/overlap_reviewer/testdata/test.1175.injected.xlsx
+++ b/overlap_reviewer/testdata/test.1175.injected.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4263,6 +4263,264 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr">
+        <is>
+          <t>00:04:46:02</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="inlineStr">
+        <is>
+          <t>00:04:48:10</t>
+        </is>
+      </c>
+      <c r="C102" s="1" t="inlineStr">
+        <is>
+          <t>Darf ich vorstellen: Bjungho Kim und Sungmin Bark.</t>
+        </is>
+      </c>
+      <c r="D102" s="1" t="inlineStr">
+        <is>
+          <t>STEDE</t>
+        </is>
+      </c>
+      <c r="E102" s="1" t="inlineStr">
+        <is>
+          <t>Darf ich vorstellen: Byung-ho Kim und Seung-min Park.</t>
+        </is>
+      </c>
+      <c r="F102" s="1" t="inlineStr">
+        <is>
+          <t>00:04:46:02</t>
+        </is>
+      </c>
+      <c r="G102" s="1" t="inlineStr">
+        <is>
+          <t>00:04:48:12</t>
+        </is>
+      </c>
+      <c r="H102" s="1" t="inlineStr"/>
+      <c r="I102" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR/PHONETIC: Byung-ho Kim → Bjungho Kim; Seung-min Park → Sungmin Bark. Original-Schreibweise nutzen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>00:04:48:14</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t>00:04:49:20</t>
+        </is>
+      </c>
+      <c r="C103" s="1" t="inlineStr">
+        <is>
+          <t>Und das ist Kinghi Tschoi.</t>
+        </is>
+      </c>
+      <c r="D103" s="1" t="inlineStr">
+        <is>
+          <t>STEDE</t>
+        </is>
+      </c>
+      <c r="E103" s="1" t="inlineStr">
+        <is>
+          <t>Und das ist Gyeong-hui Choi.</t>
+        </is>
+      </c>
+      <c r="F103" s="1" t="inlineStr">
+        <is>
+          <t>00:04:48:14</t>
+        </is>
+      </c>
+      <c r="G103" s="1" t="inlineStr">
+        <is>
+          <t>00:04:49:22</t>
+        </is>
+      </c>
+      <c r="H103" s="1" t="inlineStr"/>
+      <c r="I103" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR/PHONETIC: Gyeong-hui Choi → Kinghi Tschoi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>00:04:50:00</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="inlineStr">
+        <is>
+          <t>00:04:51:18</t>
+        </is>
+      </c>
+      <c r="C104" s="1" t="inlineStr">
+        <is>
+          <t>Pingho hier, Captain Bonnet.</t>
+        </is>
+      </c>
+      <c r="D104" s="1" t="inlineStr">
+        <is>
+          <t>BYUNG-HO</t>
+        </is>
+      </c>
+      <c r="E104" s="1" t="inlineStr">
+        <is>
+          <t>Freut mich, Captain Bonnet.</t>
+        </is>
+      </c>
+      <c r="F104" s="1" t="inlineStr">
+        <is>
+          <t>00:04:50:00</t>
+        </is>
+      </c>
+      <c r="G104" s="1" t="inlineStr">
+        <is>
+          <t>00:04:51:20</t>
+        </is>
+      </c>
+      <c r="H104" s="1" t="inlineStr"/>
+      <c r="I104" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR + NONSENSE: Byung-ho komplett falsch als Pingho; Satzanfang nicht Original. Orig: Freut mich, Captain Bonnet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>00:04:52:00</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t>00:04:54:08</t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="inlineStr">
+        <is>
+          <t>Gion wartet draußen bei Cheng Isao.</t>
+        </is>
+      </c>
+      <c r="D105" s="1" t="inlineStr">
+        <is>
+          <t>SEUNG-MIN</t>
+        </is>
+      </c>
+      <c r="E105" s="1" t="inlineStr">
+        <is>
+          <t>Ji-yeon wartet draußen bei Zheng Yi Sao.</t>
+        </is>
+      </c>
+      <c r="F105" s="1" t="inlineStr">
+        <is>
+          <t>00:04:52:00</t>
+        </is>
+      </c>
+      <c r="G105" s="1" t="inlineStr">
+        <is>
+          <t>00:04:54:10</t>
+        </is>
+      </c>
+      <c r="H105" s="1" t="inlineStr"/>
+      <c r="I105" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR: Ji-yeon → Gion; Zheng Yi Sao → Cheng Isao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr">
+        <is>
+          <t>00:04:54:12</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="inlineStr">
+        <is>
+          <t>00:04:55:22</t>
+        </is>
+      </c>
+      <c r="C106" s="1" t="inlineStr">
+        <is>
+          <t>Uschin kommt gleich, Captain.</t>
+        </is>
+      </c>
+      <c r="D106" s="1" t="inlineStr">
+        <is>
+          <t>GYEONG-HUI</t>
+        </is>
+      </c>
+      <c r="E106" s="1" t="inlineStr">
+        <is>
+          <t>Woo-jin kommt gleich, Captain.</t>
+        </is>
+      </c>
+      <c r="F106" s="1" t="inlineStr">
+        <is>
+          <t>00:04:54:12</t>
+        </is>
+      </c>
+      <c r="G106" s="1" t="inlineStr">
+        <is>
+          <t>00:04:56:00</t>
+        </is>
+      </c>
+      <c r="H106" s="1" t="inlineStr"/>
+      <c r="I106" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR/PHONETIC: Woo-jin → Uschin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr">
+        <is>
+          <t>00:04:56:02</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="inlineStr">
+        <is>
+          <t>00:04:57:16</t>
+        </is>
+      </c>
+      <c r="C107" s="1" t="inlineStr">
+        <is>
+          <t>Joey Jin, nicht wahr?</t>
+        </is>
+      </c>
+      <c r="D107" s="1" t="inlineStr">
+        <is>
+          <t>STEDE</t>
+        </is>
+      </c>
+      <c r="E107" s="1" t="inlineStr">
+        <is>
+          <t>Woo-jin Jeong, nicht wahr?</t>
+        </is>
+      </c>
+      <c r="F107" s="1" t="inlineStr">
+        <is>
+          <t>00:04:56:02</t>
+        </is>
+      </c>
+      <c r="G107" s="1" t="inlineStr">
+        <is>
+          <t>00:04:57:18</t>
+        </is>
+      </c>
+      <c r="H107" s="1" t="inlineStr"/>
+      <c r="I107" s="1" t="inlineStr">
+        <is>
+          <t>NAME_ERROR komplett falsch: Woo-jin Jeong → Joey Jin (ASR hat den Namen erfunden).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>